<commit_message>
tools: W-1 sessions re-run after the assistant fixes (modify corrects itself to 1.948 via the profile-lines warning; report carries results and the file hash; Spencer by default); audit updated
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XjjT2aBxw8gY7EFdpoUcpj
</commit_message>
<xml_diff>
--- a/docs/tutorials/files/w1_modify_after_1.xlsx
+++ b/docs/tutorials/files/w1_modify_after_1.xlsx
@@ -9023,7 +9023,7 @@
     </row>
     <row r="10" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A10" s="3">
-        <v>30.0</v>
+        <v>48.0</v>
       </c>
       <c r="B10" s="3">
         <v>24.0</v>
@@ -9071,13 +9071,13 @@
     </row>
     <row r="11" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A11" s="3">
-        <v>32.0</v>
+        <v>50.0</v>
       </c>
       <c r="B11" s="3">
         <v>24.0</v>
       </c>
       <c r="D11" s="3">
-        <v>32.0</v>
+        <v>50.0</v>
       </c>
       <c r="E11" s="3">
         <v>24.0</v>
@@ -11597,7 +11597,7 @@
         <v>24.0</v>
       </c>
       <c r="C4" s="3">
-        <v>48.0</v>
+        <v>40.0</v>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>

</xml_diff>